<commit_message>
Cambios en todos los estilos de los HTML
</commit_message>
<xml_diff>
--- a/Reporte_Tareas_2026-02-23.xlsx
+++ b/Reporte_Tareas_2026-02-23.xlsx
@@ -31,7 +31,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -48,12 +48,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="0028A745"/>
         <bgColor rgb="0028A745"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC107"/>
-        <bgColor rgb="00FFC107"/>
       </patternFill>
     </fill>
   </fills>
@@ -75,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -84,9 +78,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -454,16 +445,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -807,9 +798,9 @@
           <t>2026-02-23</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1975,16 +1966,16 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Manuel Tobio</t>
+          <t>Paula Comesaña</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Med, FGI, FFC</t>
+          <t>ACCV Jorge</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2004,13 +1995,13 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>certificadosdigitales</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
@@ -2039,22 +2030,22 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>certificadosdigitales</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Paula Comeseña</t>
+          <t>Manuel Tobio</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>AACV JORGE</t>
+          <t>Med, FGI, FFC</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2074,7 +2065,1267 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>certificadosdigitales</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>MEC</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Bryan Percy Saldivar Espinoza</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>rrhh</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Raquel Rodriguez</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>FFC</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Certificados digitales</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>certificadosdigitales</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Manuel Jimenez</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Med, FGI, FFC</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Certificados digitales</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>certificadosdigitales</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>SANP020PO</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Desactivado Scorm</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026 incidencia</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>MEC</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Miguel Ignacio López Infantozzi</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>rrhh</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>MEC</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Eva Suárez Cores</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>rrhh</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Jacobo Manuel Martínez Fernández</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>rrhh</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>MEC</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Molto Grau</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>rrhh</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>SSCG064PO</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Desactivado Scorm</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026 incidencia</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>CEC</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Víctor Bueso Martínez</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>rrhh</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SSCG064PO </t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>id=297 matriculados alumnos</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>IFCT163PO</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>id=277 matriculados tutor ver alumnos</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-09</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>ADGG020PO</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>id=287 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>COMT104PO</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>id=296 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>ADGD082PO</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>id=291 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>ADGG040PO</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>id=288 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>ADGG071PO</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>id=278 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>IFCM026PO</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>id=299 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>ADGD088PO</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>id=279 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>SSCE002PO</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>id=275 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>SSCE002PO</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>id=276 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>SSCG050PO</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>id=280 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>SANP020PO</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>id=290 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>SANP020PO</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>id=300 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>SSCG064PO</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>id=297 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>SSCG064PO</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>id=298 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>ADGD130PO</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>id=281 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>COMM002PO</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>id=289 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>ADGG072PO</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>id=272 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>ADGD066PO</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>id=294 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>ADGD162PO</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>id=286 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>SSCE002PO</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>id=273 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>ADGD318PO</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>id=283 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>ADGD290PO</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>id=284 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADGG0408 </t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Manu Jimenez - Aula virtual y encuestas</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Incidencias</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>incidencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>MF0226_3</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Grupo = L1SFC24/00096</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Campus</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>campus</t>
         </is>
       </c>
     </row>
@@ -2089,16 +3340,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
     <col width="47" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2197,9 +3448,9 @@
           <t>2026-02-23</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -2245,16 +3496,16 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Manuel Tobio</t>
+          <t>Paula Comesaña</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Med, FGI, FFC</t>
+          <t>ACCV Jorge</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -2274,13 +3525,13 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>certificadosdigitales</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -2309,22 +3560,22 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>certificadosdigitales</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Paula Comeseña</t>
+          <t>Manuel Tobio</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>AACV JORGE</t>
+          <t>Med, FGI, FFC</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -2344,7 +3595,322 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>certificadosdigitales</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Raquel Rodriguez</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>FFC</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Certificados digitales</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>certificadosdigitales</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Manuel Jimenez</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Med, FGI, FFC</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Certificados digitales</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>certificadosdigitales</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>SANP020PO</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Desactivado Scorm</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026 incidencia</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>SSCG064PO</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Desactivado Scorm</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026 incidencia</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>CEC</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Víctor Bueso Martínez</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>rrhh</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SSCG064PO </t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>id=297 matriculados alumnos</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>SANP020PO</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>id=290 matriculados, alumnos tutor ver</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADGG0408 </t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Manu Jimenez - Aula virtual y encuestas</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Incidencias</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>incidencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>MF0226_3</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Grupo = L1SFC24/00096</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Campus</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>campus</t>
         </is>
       </c>
     </row>

</xml_diff>